<commit_message>
6 cluster analysis of factoriescap_s costs 0
</commit_message>
<xml_diff>
--- a/clustering/8 subclusters (factoriescap_s (costs) 0).xlsx
+++ b/clustering/8 subclusters (factoriescap_s (costs) 0).xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12885"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -81,6 +81,8 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
     <font>
       <sz val="11"/>

</xml_diff>